<commit_message>
Final polish and accuracy fixes
</commit_message>
<xml_diff>
--- a/requirements/05_Requirements_Catalog.xlsx
+++ b/requirements/05_Requirements_Catalog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements Catalog" sheetId="1" r:id="R07b7c05349754ffb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Ra7c6868c8a14459a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements Catalog" sheetId="1" r:id="Rb77cdfcc6696402c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R40a0876f30da4d69"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -877,7 +877,7 @@
         <x:v>Display monthly requests and dispositions together over time.</x:v>
       </x:c>
       <x:c r="D19" s="36" t="str">
-        <x:v>Supports direct comparison of intake and completion activity.</x:v>
+        <x:v>Supports direct comparison of intake and disposition activity.</x:v>
       </x:c>
       <x:c r="E19" s="36" t="str">
         <x:v>Must</x:v>
@@ -1019,7 +1019,7 @@
         <x:v>Functional</x:v>
       </x:c>
       <x:c r="C24" s="36" t="str">
-        <x:v>Preserve the analytical distinction between open requests and completed/dispositioned records.</x:v>
+        <x:v>Preserve the analytical distinction between open requests and dispositioned records.</x:v>
       </x:c>
       <x:c r="D24" s="36" t="str">
         <x:v>Prevents backlog metrics from being confused with total historical volume.</x:v>
@@ -1299,7 +1299,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R082e687238be4f4c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dc76cdd59d146e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>